<commit_message>
correcting misc_format_check to return a warning for VALUES being the last column of the data dictionary; addition of new functions to documentation; polishing documentation
</commit_message>
<xml_diff>
--- a/inst/extdata/Functions.xlsx
+++ b/inst/extdata/Functions.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/law145/Desktop/packages/dbGaPCheckup/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D64A49-C543-8A43-80E3-E4961C1CA101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FF69CC-C7DD-9241-AA5D-76A1B750F026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="39780" yWindow="2300" windowWidth="28040" windowHeight="16940" xr2:uid="{0EA5F04A-9331-CF41-B115-F8A4A1753AE3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="76">
   <si>
     <t>dictionary_search</t>
   </si>
@@ -246,6 +246,24 @@
   </si>
   <si>
     <t>Checks miscellaneous dbGaP formatting requirements to ensure (1) no empty variable names; (2) no duplicate variable names; (3) variable names do not contain "dbgap"; (4) there are no duplicate column names in the dictionary; and (5) column names falling after `VALUES` column are unnamed.</t>
+  </si>
+  <si>
+    <t>ascii_cleaner</t>
+  </si>
+  <si>
+    <t>Scans a data frame for common problematic characters and returns a cleaned version by: converting smart quotes (e.g., curved) to ASCII quotes (e.g., " and '); replacing accented characters with ASCII equivalents (e.g., e, n); removing newline and carriage return characters (that create line breaks)</t>
+  </si>
+  <si>
+    <t>duplicate_id_check</t>
+  </si>
+  <si>
+    <t>ascii_check</t>
+  </si>
+  <si>
+    <t>Scans for non-ASCII characters (e.g., with accents) and newline and carriage return characters (e.g., line breaks)</t>
+  </si>
+  <si>
+    <t>Checks for duplicated SUBJECT_ID values are present in the dataset (while expected/allowable in longitudinal data, it may indicate an error in cross-sectional submissions)</t>
   </si>
 </sst>
 </file>
@@ -320,9 +338,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -360,7 +378,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -466,7 +484,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -608,7 +626,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -616,7 +634,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83CC6E43-0634-6E40-A686-F511C6932B48}">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.83203125" bestFit="1" customWidth="1"/>
@@ -698,303 +716,339 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="1"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="B13" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="D13" s="1"/>
+    </row>
+    <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="B14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="1"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="1"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B19" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="D19" s="1"/>
     </row>
     <row r="20" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D20" s="1"/>
     </row>
     <row r="21" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="1"/>
+    </row>
+    <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D25" s="1"/>
+    </row>
+    <row r="26" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D26" s="1"/>
+    </row>
+    <row r="27" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" s="1"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D26" s="1"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="D27" s="1"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D28" s="1"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D29" s="1"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="D30" s="1"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D31" s="1"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="1"/>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D33" s="1"/>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C34" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D31" s="1"/>
+      <c r="D34" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updating values_check to check that there are no duplicated MEANINGs within a data dictionary row (e.g., 0=FEMALE, 1=FEMALE)
</commit_message>
<xml_diff>
--- a/inst/extdata/Functions.xlsx
+++ b/inst/extdata/Functions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/law145/Desktop/packages/dbGaPCheckup/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FF69CC-C7DD-9241-AA5D-76A1B750F026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BCDD1B6-E13C-5642-B4C0-0B6F3806FB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39780" yWindow="2300" windowWidth="28040" windowHeight="16940" xr2:uid="{0EA5F04A-9331-CF41-B115-F8A4A1753AE3}"/>
+    <workbookView xWindow="10020" yWindow="1540" windowWidth="28040" windowHeight="16940" xr2:uid="{0EA5F04A-9331-CF41-B115-F8A4A1753AE3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -176,9 +176,6 @@
     <t>Checks for NA values in the data set and, if NA values are present, also checks for an encoded NA value=meaning description.</t>
   </si>
   <si>
-    <t>Checks for potential errors in the VALUES columns by ensuring (1) required format of `VALUE=MEANING` (e.g., 0=No or 1=Yes); (2) no leading/trailing spaces near the equals sign (e.g., 0=No vs. 0 = No); (3) all variables of TYPE encoded have VALUES entries; and (4) all variables with VALUES entries are listed as TYPE encoded.</t>
-  </si>
-  <si>
     <t>Checks for variables that have values exceeding the listed MIN or MAX.</t>
   </si>
   <si>
@@ -264,6 +261,9 @@
   </si>
   <si>
     <t>Checks for duplicated SUBJECT_ID values are present in the dataset (while expected/allowable in longitudinal data, it may indicate an error in cross-sectional submissions)</t>
+  </si>
+  <si>
+    <t>Checks for potential errors in the VALUES columns by ensuring (1) required format of `VALUE=MEANING` (e.g., 0=Yes or 1=No) AND ensuring there is only one equals sign per cell; (2) no leading/trailing spaces near the equals sign; (3) all variables of TYPE encoded have VALUES entries; (4) all variables with VALUES entries are listed as TYPE encoded; and (5) there are no duplicated MEANINGs (e.g., 1=Yes; 2=Yes) within the same variable</t>
   </si>
 </sst>
 </file>
@@ -686,7 +686,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D4" s="1"/>
     </row>
@@ -710,19 +710,19 @@
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D7" s="1"/>
     </row>
@@ -734,7 +734,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D8" s="1"/>
     </row>
@@ -770,7 +770,7 @@
         <v>2</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="D11" s="1"/>
     </row>
@@ -806,7 +806,7 @@
         <v>2</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D14" s="1"/>
     </row>
@@ -830,19 +830,19 @@
         <v>2</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="D17" s="1"/>
     </row>
@@ -854,7 +854,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D18" s="1"/>
     </row>
@@ -866,91 +866,91 @@
         <v>16</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D19" s="1"/>
     </row>
     <row r="20" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D20" s="1"/>
     </row>
     <row r="21" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="C22" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D24" s="1"/>
     </row>
     <row r="25" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="D26" s="1"/>
     </row>
@@ -962,7 +962,7 @@
         <v>33</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D27" s="1"/>
     </row>
@@ -998,7 +998,7 @@
         <v>21</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D30" s="1"/>
     </row>
@@ -1031,7 +1031,7 @@
         <v>38</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>28</v>
@@ -1043,7 +1043,7 @@
         <v>39</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>40</v>

</xml_diff>